<commit_message>
modificaciones proceso nuevo cliente
</commit_message>
<xml_diff>
--- a/assets/procesos/nuevos-clientes-instalacion/matrices-responsabilidades.xlsx
+++ b/assets/procesos/nuevos-clientes-instalacion/matrices-responsabilidades.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,8 +62,13 @@
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +110,31 @@
         <fgColor rgb="FFBDD7EE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6E0B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -133,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -176,10 +206,72 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FCE4B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -541,7 +633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" style="13" min="1" max="1"/>
@@ -549,7 +641,9 @@
     <col width="22" customWidth="1" style="13" min="3" max="3"/>
     <col width="16" customWidth="1" style="13" min="4" max="4"/>
     <col width="60.6640625" customWidth="1" style="13" min="5" max="5"/>
-    <col width="26" customWidth="1" style="13" min="6" max="6"/>
+    <col width="16" customWidth="1" style="13" min="6" max="6"/>
+    <col width="24" customWidth="1" style="13" min="7" max="7"/>
+    <col width="50" customWidth="1" style="13" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.4" customHeight="1" s="13">
@@ -569,7 +663,7 @@
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>Referencias: Verde = resuelto   |   Ámbar = a definir   |   N° = mismo número de hito que la hoja Responsabilidades</t>
+          <t>Referencias: Ámbar en área/medio = a definir   |   N° = mismo número de hito que la hoja Responsabilidades</t>
         </is>
       </c>
     </row>
@@ -602,11 +696,21 @@
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>Estado</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="26.4" customHeight="1" s="13">
+          <t>Estado de validación</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="39.6" customHeight="1" s="13">
       <c r="A5" s="2" t="n">
         <v>1</v>
       </c>
@@ -630,228 +734,369 @@
           <t>Confirmación de la compra y próximos pasos (que Instalaciones se va a poner en contacto)</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Resuelto</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="26.4" customHeight="1" s="13">
+      <c r="F5" s="26" t="inlineStr">
+        <is>
+          <t>Validado</t>
+        </is>
+      </c>
+      <c r="G5" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Et. 6 · R1</t>
+        </is>
+      </c>
+      <c r="H5" s="17" t="inlineStr"/>
+    </row>
+    <row r="6" ht="52" customHeight="1" s="13">
       <c r="A6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Gestión del cobro (presentación, medio de pago y aviso de vencimiento)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Atención al Cliente</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp (mensaje automático GHL) y telefónico</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Presentación del área, medio de pago acordado y vencimiento del presupuesto</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="G6" s="17" t="inlineStr">
+        <is>
+          <t>R2 (30/09)</t>
+        </is>
+      </c>
+      <c r="H6" s="17" t="inlineStr">
+        <is>
+          <t>Puntos abiertos en R2: datos mínimos del traspaso, protocolo de contacto sin respuesta, vigencia del presupuesto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="39.6" customHeight="1" s="13">
+      <c r="A7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Coordinación de la fecha de instalación</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
         <is>
           <t>A DEFINIR</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Fecha y horario en que se realizará la instalación</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="26.4" customHeight="1" s="13">
-      <c r="A7" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Consultas del cliente mientras no hay fecha confirmada</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Estado de la coordinación de su instalación</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>A definir</t>
+      <c r="F7" s="27" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="G7" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Et. 9 · R1 (tratado, sin cierre)</t>
+        </is>
+      </c>
+      <c r="H7" s="17" t="inlineStr">
+        <is>
+          <t>Incluye informar el tiempo estimado del trabajo.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="39.6" customHeight="1" s="13">
       <c r="A8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Consultas del cliente mientras no hay fecha confirmada</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>A DEFINIR</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Estado de la coordinación de su instalación</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="G8" s="17" t="inlineStr">
+        <is>
+          <t>Inferido de Et. 9 · R1 (tratado, sin cierre)</t>
+        </is>
+      </c>
+      <c r="H8" s="17" t="inlineStr">
+        <is>
+          <t>No surge del relevamiento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="39.6" customHeight="1" s="13">
+      <c r="A9" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Cierre de la instalación y firma del acta de conformidad</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Instalaciones</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Presencial</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Conformidad del trabajo realizado y detalle de pendientes, si los hay</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>A definir si comunica con claridad la activación del sistema</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="26.4" customHeight="1" s="13">
-      <c r="A9" s="2" t="n">
+      <c r="F9" s="27" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="G9" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Et. 10 · R1</t>
+        </is>
+      </c>
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>A definir si comunica con claridad la activación del sistema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="39.6" customHeight="1" s="13">
+      <c r="A10" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Comunicación de finalización / activación del sistema</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Que el sistema quedó activo y operativo</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Et. 10 · R1 (tratado, sin cierre)</t>
+        </is>
+      </c>
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t>Se comunica al cierre de la instalación (alta en la central y capacitación).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1" s="13">
+      <c r="A11" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Contacto de Posventa (control de calidad y satisfacción)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Posventa</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Canal de posventa</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Encuesta de satisfacción y relevamiento de pendientes</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="G11" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Control de calidad posventa · R1</t>
+        </is>
+      </c>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>Momento exacto de inicio a definir. La bienvenida no es parte de este contacto: es la etapa 8, a cargo de Atención al Cliente (definido 06/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="39.6" customHeight="1" s="13">
+      <c r="A12" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Reclamo o consulta posterior a la instalación</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>Posventa (período inicial) / Servicio Técnico (técnicos)</t>
+        </is>
+      </c>
+      <c r="D12" s="20" t="inlineStr">
         <is>
           <t>A DEFINIR</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Según el tipo de solicitud (comercial / técnica / servicio)</t>
+        </is>
+      </c>
+      <c r="F12" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Control de calidad posventa / Et. 12</t>
+        </is>
+      </c>
+      <c r="H12" s="17" t="inlineStr">
+        <is>
+          <t>No define reclamos comerciales ni de servicio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="39.6" customHeight="1" s="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Seguimiento de un caso derivado a Servicio Técnico</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>Servicio Técnico</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
         <is>
           <t>A DEFINIR</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Que el sistema quedó activo y operativo</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="26.4" customHeight="1" s="13">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Contacto de Posventa (control de calidad y satisfacción)</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Posventa</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Canal de posventa</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>Encuesta de satisfacción y relevamiento de pendientes</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>Resuelto en general; momento exacto de inicio a definir</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="26.4" customHeight="1" s="13">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Reclamo o consulta posterior a la instalación</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>A DEFINIR según tipo de solicitud</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Según el tipo de solicitud (comercial / técnica / servicio)</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="26.4" customHeight="1" s="13">
-      <c r="A12" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Seguimiento de un caso derivado a Servicio Técnico</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Estado de la resolución y plazo estimado</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>A definir (incluye SLA)</t>
+      <c r="F13" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Et. 12</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>Cierra el reclamo con la conformidad del cliente. SLA a definir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15" ht="30" customHeight="1" s="13">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>Estado de validación: Pendiente = responsable tomado del relevamiento (Proceso de Venta y Atención por Áreas), sin revisar con las áreas   |   En proceso = en revisión con las áreas, con puntos abiertos   |   Validado = confirmado por las áreas involucradas</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+  <mergeCells count="4">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A15:H15"/>
   </mergeCells>
+  <conditionalFormatting sqref="F5:F13">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Pendiente"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"En proceso"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Validado"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="F5:F13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pendiente,En proceso,Validado"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -863,7 +1108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" style="13" min="1" max="1"/>
@@ -873,7 +1118,9 @@
     <col width="14" customWidth="1" style="13" min="5" max="5"/>
     <col width="16" customWidth="1" style="13" min="6" max="6"/>
     <col width="13" customWidth="1" style="13" min="7" max="7"/>
-    <col width="30" customWidth="1" style="13" min="8" max="8"/>
+    <col width="16" customWidth="1" style="13" min="8" max="8"/>
+    <col width="24" customWidth="1" style="13" min="9" max="9"/>
+    <col width="55" customWidth="1" style="13" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.05" customHeight="1" s="13">
@@ -935,11 +1182,21 @@
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>Estado</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>Estado de validación</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="39.6" customHeight="1" s="13">
       <c r="A5" s="2" t="n">
         <v>1</v>
       </c>
@@ -973,11 +1230,17 @@
           <t>No participa</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>Resuelto</t>
-        </is>
-      </c>
+      <c r="H5" s="26" t="inlineStr">
+        <is>
+          <t>Validado</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Et. 6 · R1</t>
+        </is>
+      </c>
+      <c r="J5" s="17" t="inlineStr"/>
     </row>
     <row r="6" ht="39.6" customHeight="1" s="13">
       <c r="A6" s="2" t="n">
@@ -1013,13 +1276,23 @@
           <t>No participa</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Resuelto</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="26.4" customHeight="1" s="13">
+      <c r="H6" s="26" t="inlineStr">
+        <is>
+          <t>Validado</t>
+        </is>
+      </c>
+      <c r="I6" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Et. 7 · R1 · R2</t>
+        </is>
+      </c>
+      <c r="J6" s="17" t="inlineStr">
+        <is>
+          <t>Datos mínimos del traspaso a completar (R2). Definido 06/10: incluyen la forma de pago, para saber cuándo esperar el primer cobro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="39.6" customHeight="1" s="13">
       <c r="A7" s="2" t="n">
         <v>3</v>
       </c>
@@ -1028,38 +1301,48 @@
           <t>Coordinación de la fecha de instalación con el cliente</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="26.4" customHeight="1" s="13">
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="G7" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="H7" s="27" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Et. 9 · R1 (tratado, sin cierre)</t>
+        </is>
+      </c>
+      <c r="J7" s="17" t="inlineStr">
+        <is>
+          <t>Instalaciones contacta al cliente para acordar día, horario y duración estimada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="39.6" customHeight="1" s="13">
       <c r="A8" s="2" t="n">
         <v>4</v>
       </c>
@@ -1068,38 +1351,48 @@
           <t>Atención de consultas del cliente mientras no hay fecha confirmada</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
+      <c r="C8" s="25" t="inlineStr">
+        <is>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="H8" s="27" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="I8" s="17" t="inlineStr">
+        <is>
+          <t>Inferido de Et. 9 · R1 (tratado, sin cierre)</t>
+        </is>
+      </c>
+      <c r="J8" s="17" t="inlineStr">
+        <is>
+          <t>El relevamiento no lo menciona; se asigna a Instalaciones por ser dueña de la coordinación. Hoy estas consultas llegan a Ventas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="39.6" customHeight="1" s="13">
       <c r="A9" s="2" t="n">
         <v>5</v>
       </c>
@@ -1133,13 +1426,19 @@
           <t>No participa</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Resuelto</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="26.4" customHeight="1" s="13">
+      <c r="H9" s="26" t="inlineStr">
+        <is>
+          <t>Validado</t>
+        </is>
+      </c>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Et. 10 · R1</t>
+        </is>
+      </c>
+      <c r="J9" s="17" t="inlineStr"/>
+    </row>
+    <row r="10" ht="39.6" customHeight="1" s="13">
       <c r="A10" s="2" t="n">
         <v>6</v>
       </c>
@@ -1173,13 +1472,19 @@
           <t>No participa</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>Resuelto</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="26.4" customHeight="1" s="13">
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>Validado</t>
+        </is>
+      </c>
+      <c r="I10" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Et. 10 · R1</t>
+        </is>
+      </c>
+      <c r="J10" s="17" t="inlineStr"/>
+    </row>
+    <row r="11" ht="39.6" customHeight="1" s="13">
       <c r="A11" s="2" t="n">
         <v>7</v>
       </c>
@@ -1188,38 +1493,48 @@
           <t>Registro de pendientes en el acta con responsable y plazo asignado</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>A definir (hoy el acta no asigna responsable ni plazo)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="26.4" customHeight="1" s="13">
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="E11" s="24" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="F11" s="25" t="inlineStr">
+        <is>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="G11" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="H11" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>Inferido de Et. 10</t>
+        </is>
+      </c>
+      <c r="J11" s="17" t="inlineStr">
+        <is>
+          <t>Hoy el acta no asigna responsable ni plazo. Instalaciones cierra el acta; la asignación de responsable/plazo no está relevada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="39.6" customHeight="1" s="13">
       <c r="A12" s="2" t="n">
         <v>8</v>
       </c>
@@ -1228,38 +1543,48 @@
           <t>Comunicación de finalización / activación del sistema al cliente</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="D12" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="E12" s="24" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="F12" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="G12" s="25" t="inlineStr">
+        <is>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="H12" s="27" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="I12" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Et. 10 / Control de calidad posventa · R1 (tratado, sin cierre)</t>
+        </is>
+      </c>
+      <c r="J12" s="17" t="inlineStr">
+        <is>
+          <t>Instalaciones da de alta el sistema en la central y capacita al cliente; Posventa valida luego el funcionamiento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1" s="13">
       <c r="A13" s="2" t="n">
         <v>9</v>
       </c>
@@ -1293,13 +1618,23 @@
           <t>Responsable</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Resuelto</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="26.4" customHeight="1" s="13">
+      <c r="H13" s="26" t="inlineStr">
+        <is>
+          <t>Validado</t>
+        </is>
+      </c>
+      <c r="I13" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Control de calidad posventa · R1</t>
+        </is>
+      </c>
+      <c r="J13" s="17" t="inlineStr">
+        <is>
+          <t>La bienvenida es la etapa 8, a cargo de Atención al Cliente (antes de la instalación). Este hito es el control de calidad posterior a la instalación (Posventa).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="39.6" customHeight="1" s="13">
       <c r="A14" s="2" t="n">
         <v>10</v>
       </c>
@@ -1308,38 +1643,48 @@
           <t>Clasificación y canalización de reclamos según tipo (comercial / técnico / servicio)</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="26.4" customHeight="1" s="13">
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="D14" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="E14" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="F14" s="25" t="inlineStr">
+        <is>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="G14" s="24" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="H14" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I14" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Control de calidad posventa / Et. 12</t>
+        </is>
+      </c>
+      <c r="J14" s="17" t="inlineStr">
+        <is>
+          <t>Posventa canaliza a Servicio Técnico las fallas del período inicial. El relevamiento no define reclamos comerciales ni de servicio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="39.6" customHeight="1" s="13">
       <c r="A15" s="2" t="n">
         <v>11</v>
       </c>
@@ -1373,13 +1718,23 @@
           <t>A DEFINIR</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="26.4" customHeight="1" s="13">
+      <c r="H15" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I15" s="17" t="inlineStr">
+        <is>
+          <t>No relevado</t>
+        </is>
+      </c>
+      <c r="J15" s="17" t="inlineStr">
+        <is>
+          <t>No surge del relevamiento; definir con Instalaciones, Servicio Técnico y Posventa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="39.6" customHeight="1" s="13">
       <c r="A16" s="2" t="n">
         <v>12</v>
       </c>
@@ -1413,13 +1768,23 @@
           <t>Apoya</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>A definir (SLA sin definir)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="26.4" customHeight="1" s="13">
+      <c r="H16" s="27" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="I16" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Et. 12 · R1</t>
+        </is>
+      </c>
+      <c r="J16" s="17" t="inlineStr">
+        <is>
+          <t>Responsables definidos; falta definir el SLA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="39.6" customHeight="1" s="13">
       <c r="A17" s="2" t="n">
         <v>13</v>
       </c>
@@ -1453,18 +1818,49 @@
           <t>Apoya</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>Resuelto</t>
+      <c r="H17" s="26" t="inlineStr">
+        <is>
+          <t>Validado</t>
+        </is>
+      </c>
+      <c r="I17" s="17" t="inlineStr">
+        <is>
+          <t>Relevamiento Et. 14 · R1</t>
+        </is>
+      </c>
+      <c r="J17" s="17" t="inlineStr"/>
+    </row>
+    <row r="18"/>
+    <row r="19" ht="30" customHeight="1" s="13">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>Estado de validación: Pendiente = responsable tomado del relevamiento (Proceso de Venta y Atención por Áreas), sin revisar con las áreas   |   En proceso = en revisión con las áreas, con puntos abiertos   |   Validado = confirmado por las áreas involucradas</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+  <mergeCells count="4">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A19:J19"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
+  <conditionalFormatting sqref="H5:H17">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Pendiente"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"En proceso"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Validado"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H5:H17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pendiente,En proceso,Validado"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Modificaciones relevamiento porceso nuevo cliente
</commit_message>
<xml_diff>
--- a/assets/procesos/nuevos-clientes-instalacion/matrices-responsabilidades.xlsx
+++ b/assets/procesos/nuevos-clientes-instalacion/matrices-responsabilidades.xlsx
@@ -701,7 +701,7 @@
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>Fuente</t>
+          <t>Etapas del relevamiento</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
@@ -734,17 +734,21 @@
           <t>Confirmación de la compra y próximos pasos (que Instalaciones se va a poner en contacto)</t>
         </is>
       </c>
-      <c r="F5" s="26" t="inlineStr">
-        <is>
-          <t>Validado</t>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Et. 6 · R1</t>
-        </is>
-      </c>
-      <c r="H5" s="17" t="inlineStr"/>
+          <t>1 a 6</t>
+        </is>
+      </c>
+      <c r="H5" s="17" t="inlineStr">
+        <is>
+          <t>Reuniones: R1.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="52" customHeight="1" s="13">
       <c r="A6" s="2" t="n">
@@ -777,12 +781,12 @@
       </c>
       <c r="G6" s="17" t="inlineStr">
         <is>
-          <t>R2 (30/09)</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H6" s="17" t="inlineStr">
         <is>
-          <t>Puntos abiertos en R2: datos mínimos del traspaso, protocolo de contacto sin respuesta, vigencia del presupuesto.</t>
+          <t>Puntos abiertos en R2: datos mínimos del traspaso, protocolo de contacto sin respuesta, vigencia del presupuesto. Reuniones: R1 · R2.</t>
         </is>
       </c>
     </row>
@@ -810,19 +814,19 @@
           <t>Fecha y horario en que se realizará la instalación</t>
         </is>
       </c>
-      <c r="F7" s="27" t="inlineStr">
-        <is>
-          <t>En proceso</t>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Et. 9 · R1 (tratado, sin cierre)</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H7" s="17" t="inlineStr">
         <is>
-          <t>Incluye informar el tiempo estimado del trabajo.</t>
+          <t>Incluye informar el tiempo estimado del trabajo. Reuniones: R1 (tratado, sin cierre).</t>
         </is>
       </c>
     </row>
@@ -850,19 +854,19 @@
           <t>Estado de la coordinación de su instalación</t>
         </is>
       </c>
-      <c r="F8" s="27" t="inlineStr">
-        <is>
-          <t>En proceso</t>
+      <c r="F8" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
-          <t>Inferido de Et. 9 · R1 (tratado, sin cierre)</t>
+          <t>9 (inferido)</t>
         </is>
       </c>
       <c r="H8" s="17" t="inlineStr">
         <is>
-          <t>No surge del relevamiento.</t>
+          <t>No surge del relevamiento. Reuniones: R1 (tratado, sin cierre).</t>
         </is>
       </c>
     </row>
@@ -890,14 +894,14 @@
           <t>Conformidad del trabajo realizado y detalle de pendientes, si los hay</t>
         </is>
       </c>
-      <c r="F9" s="27" t="inlineStr">
-        <is>
-          <t>En proceso</t>
+      <c r="F9" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Et. 10 · R1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H9" s="17" t="inlineStr">
@@ -930,19 +934,19 @@
           <t>Que el sistema quedó activo y operativo</t>
         </is>
       </c>
-      <c r="F10" s="27" t="inlineStr">
-        <is>
-          <t>En proceso</t>
+      <c r="F10" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G10" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Et. 10 · R1 (tratado, sin cierre)</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H10" s="17" t="inlineStr">
         <is>
-          <t>Se comunica al cierre de la instalación (alta en la central y capacitación).</t>
+          <t>Se comunica al cierre de la instalación (alta en la central y capacitación). Reuniones: R1 (tratado, sin cierre).</t>
         </is>
       </c>
     </row>
@@ -970,14 +974,14 @@
           <t>Encuesta de satisfacción y relevamiento de pendientes</t>
         </is>
       </c>
-      <c r="F11" s="27" t="inlineStr">
-        <is>
-          <t>En proceso</t>
+      <c r="F11" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Control de calidad posventa · R1</t>
+          <t>Control de calidad posventa</t>
         </is>
       </c>
       <c r="H11" s="17" t="inlineStr">
@@ -1017,7 +1021,7 @@
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Control de calidad posventa / Et. 12</t>
+          <t>Control de calidad posventa / 12</t>
         </is>
       </c>
       <c r="H12" s="17" t="inlineStr">
@@ -1057,7 +1061,7 @@
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Et. 12</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H13" s="17" t="inlineStr">
@@ -1070,7 +1074,7 @@
     <row r="15" ht="30" customHeight="1" s="13">
       <c r="A15" s="22" t="inlineStr">
         <is>
-          <t>Estado de validación: Pendiente = responsable tomado del relevamiento (Proceso de Venta y Atención por Áreas), sin revisar con las áreas   |   En proceso = en revisión con las áreas, con puntos abiertos   |   Validado = confirmado por las áreas involucradas</t>
+          <t>Estado de validación: Pendiente = relevamiento del hito aún no iniciado (responsable tomado del documento de relevamiento)   |   En proceso = relevamiento en curso: reuniones con las áreas y minutas   |   Validado = relevamiento realizado, reuniones con sus minutas y validación formal del sector</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1191,7 @@
       </c>
       <c r="I4" s="1" t="inlineStr">
         <is>
-          <t>Fuente</t>
+          <t>Etapas del relevamiento</t>
         </is>
       </c>
       <c r="J4" s="1" t="inlineStr">
@@ -1230,17 +1234,21 @@
           <t>No participa</t>
         </is>
       </c>
-      <c r="H5" s="26" t="inlineStr">
-        <is>
-          <t>Validado</t>
+      <c r="H5" s="27" t="inlineStr">
+        <is>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="I5" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Et. 6 · R1</t>
-        </is>
-      </c>
-      <c r="J5" s="17" t="inlineStr"/>
+          <t>1 a 6</t>
+        </is>
+      </c>
+      <c r="J5" s="17" t="inlineStr">
+        <is>
+          <t>Reuniones: R1.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="39.6" customHeight="1" s="13">
       <c r="A6" s="2" t="n">
@@ -1276,19 +1284,19 @@
           <t>No participa</t>
         </is>
       </c>
-      <c r="H6" s="26" t="inlineStr">
-        <is>
-          <t>Validado</t>
+      <c r="H6" s="27" t="inlineStr">
+        <is>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="I6" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Et. 7 · R1 · R2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J6" s="17" t="inlineStr">
         <is>
-          <t>Datos mínimos del traspaso a completar (R2). Definido 06/10: incluyen la forma de pago, para saber cuándo esperar el primer cobro.</t>
+          <t>Datos mínimos del traspaso a completar (R2). Definido 06/10: incluyen la forma de pago, para saber cuándo esperar el primer cobro. Reuniones: R1 · R2.</t>
         </is>
       </c>
     </row>
@@ -1326,19 +1334,19 @@
           <t>No participa</t>
         </is>
       </c>
-      <c r="H7" s="27" t="inlineStr">
-        <is>
-          <t>En proceso</t>
+      <c r="H7" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="I7" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Et. 9 · R1 (tratado, sin cierre)</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J7" s="17" t="inlineStr">
         <is>
-          <t>Instalaciones contacta al cliente para acordar día, horario y duración estimada.</t>
+          <t>Instalaciones contacta al cliente para acordar día, horario y duración estimada. Reuniones: R1 (tratado, sin cierre).</t>
         </is>
       </c>
     </row>
@@ -1376,19 +1384,19 @@
           <t>No participa</t>
         </is>
       </c>
-      <c r="H8" s="27" t="inlineStr">
-        <is>
-          <t>En proceso</t>
+      <c r="H8" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="I8" s="17" t="inlineStr">
         <is>
-          <t>Inferido de Et. 9 · R1 (tratado, sin cierre)</t>
+          <t>9 (inferido)</t>
         </is>
       </c>
       <c r="J8" s="17" t="inlineStr">
         <is>
-          <t>El relevamiento no lo menciona; se asigna a Instalaciones por ser dueña de la coordinación. Hoy estas consultas llegan a Ventas.</t>
+          <t>El relevamiento no lo menciona; se asigna a Instalaciones por ser dueña de la coordinación. Hoy estas consultas llegan a Ventas. Reuniones: R1 (tratado, sin cierre).</t>
         </is>
       </c>
     </row>
@@ -1426,17 +1434,17 @@
           <t>No participa</t>
         </is>
       </c>
-      <c r="H9" s="26" t="inlineStr">
-        <is>
-          <t>Validado</t>
+      <c r="H9" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="I9" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Et. 10 · R1</t>
-        </is>
-      </c>
-      <c r="J9" s="17" t="inlineStr"/>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J9" s="17" t="n"/>
     </row>
     <row r="10" ht="39.6" customHeight="1" s="13">
       <c r="A10" s="2" t="n">
@@ -1472,17 +1480,17 @@
           <t>No participa</t>
         </is>
       </c>
-      <c r="H10" s="26" t="inlineStr">
-        <is>
-          <t>Validado</t>
+      <c r="H10" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="I10" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Et. 10 · R1</t>
-        </is>
-      </c>
-      <c r="J10" s="17" t="inlineStr"/>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J10" s="17" t="n"/>
     </row>
     <row r="11" ht="39.6" customHeight="1" s="13">
       <c r="A11" s="2" t="n">
@@ -1525,7 +1533,7 @@
       </c>
       <c r="I11" s="17" t="inlineStr">
         <is>
-          <t>Inferido de Et. 10</t>
+          <t>10 (inferido)</t>
         </is>
       </c>
       <c r="J11" s="17" t="inlineStr">
@@ -1568,19 +1576,19 @@
           <t>Informado</t>
         </is>
       </c>
-      <c r="H12" s="27" t="inlineStr">
-        <is>
-          <t>En proceso</t>
+      <c r="H12" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Et. 10 / Control de calidad posventa · R1 (tratado, sin cierre)</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J12" s="17" t="inlineStr">
         <is>
-          <t>Instalaciones da de alta el sistema en la central y capacita al cliente; Posventa valida luego el funcionamiento.</t>
+          <t>Instalaciones da de alta el sistema en la central y capacita al cliente; Posventa valida luego el funcionamiento. Reuniones: R1 (tratado, sin cierre).</t>
         </is>
       </c>
     </row>
@@ -1618,14 +1626,14 @@
           <t>Responsable</t>
         </is>
       </c>
-      <c r="H13" s="26" t="inlineStr">
-        <is>
-          <t>Validado</t>
+      <c r="H13" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="I13" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Control de calidad posventa · R1</t>
+          <t>Control de calidad posventa</t>
         </is>
       </c>
       <c r="J13" s="17" t="inlineStr">
@@ -1675,7 +1683,7 @@
       </c>
       <c r="I14" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Control de calidad posventa / Et. 12</t>
+          <t>Control de calidad posventa / 12</t>
         </is>
       </c>
       <c r="J14" s="17" t="inlineStr">
@@ -1725,7 +1733,7 @@
       </c>
       <c r="I15" s="17" t="inlineStr">
         <is>
-          <t>No relevado</t>
+          <t>— (no relevado)</t>
         </is>
       </c>
       <c r="J15" s="17" t="inlineStr">
@@ -1768,14 +1776,14 @@
           <t>Apoya</t>
         </is>
       </c>
-      <c r="H16" s="27" t="inlineStr">
-        <is>
-          <t>En proceso</t>
+      <c r="H16" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="I16" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Et. 12 · R1</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J16" s="17" t="inlineStr">
@@ -1818,23 +1826,23 @@
           <t>Apoya</t>
         </is>
       </c>
-      <c r="H17" s="26" t="inlineStr">
-        <is>
-          <t>Validado</t>
+      <c r="H17" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="I17" s="17" t="inlineStr">
         <is>
-          <t>Relevamiento Et. 14 · R1</t>
-        </is>
-      </c>
-      <c r="J17" s="17" t="inlineStr"/>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="J17" s="17" t="n"/>
     </row>
     <row r="18"/>
     <row r="19" ht="30" customHeight="1" s="13">
       <c r="A19" s="22" t="inlineStr">
         <is>
-          <t>Estado de validación: Pendiente = responsable tomado del relevamiento (Proceso de Venta y Atención por Áreas), sin revisar con las áreas   |   En proceso = en revisión con las áreas, con puntos abiertos   |   Validado = confirmado por las áreas involucradas</t>
+          <t>Estado de validación: Pendiente = relevamiento del hito aún no iniciado (responsable tomado del documento de relevamiento)   |   En proceso = relevamiento en curso: reuniones con las áreas y minutas   |   Validado = relevamiento realizado, reuniones con sus minutas y validación formal del sector</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Modificaciones proceso nuevos cliente
</commit_message>
<xml_diff>
--- a/assets/procesos/nuevos-clientes-instalacion/matrices-responsabilidades.xlsx
+++ b/assets/procesos/nuevos-clientes-instalacion/matrices-responsabilidades.xlsx
@@ -981,7 +981,7 @@
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>Control de calidad posventa</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H11" s="17" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>Control de calidad posventa / 12</t>
+          <t>11 / 13</t>
         </is>
       </c>
       <c r="H12" s="17" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H13" s="17" t="inlineStr">
@@ -1633,12 +1633,12 @@
       </c>
       <c r="I13" s="17" t="inlineStr">
         <is>
-          <t>Control de calidad posventa</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J13" s="17" t="inlineStr">
         <is>
-          <t>La bienvenida es la etapa 8, a cargo de Atención al Cliente (antes de la instalación). Este hito es el control de calidad posterior a la instalación (Posventa).</t>
+          <t>La bienvenida es la etapa 8, a cargo de Atención al Cliente (antes de la instalación). Este hito corresponde a la etapa 11, control de calidad posterior a la instalación (Posventa).</t>
         </is>
       </c>
     </row>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="I14" s="17" t="inlineStr">
         <is>
-          <t>Control de calidad posventa / 12</t>
+          <t>11 / 13</t>
         </is>
       </c>
       <c r="J14" s="17" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="I16" s="17" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J16" s="17" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="I17" s="17" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J17" s="17" t="n"/>

</xml_diff>

<commit_message>
Modificaion informe de MKT
</commit_message>
<xml_diff>
--- a/assets/procesos/nuevos-clientes-instalacion/matrices-responsabilidades.xlsx
+++ b/assets/procesos/nuevos-clientes-instalacion/matrices-responsabilidades.xlsx
@@ -68,7 +68,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -135,6 +135,11 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -163,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -243,6 +248,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -633,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" style="13" min="1" max="1"/>
@@ -1030,49 +1038,89 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="39.6" customHeight="1" s="13">
+    <row r="13" ht="40" customHeight="1" s="13">
       <c r="A13" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Escalación de un pendiente del acta no resuelto en plazo</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>Posventa</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>A DEFINIR</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Que el pendiente fue escalado, quién lo resuelve y el nuevo plazo; luego, confirmación del cierre</t>
+        </is>
+      </c>
+      <c r="F13" s="28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>11 (excepción posterior a la 10)</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>Propuesta 07/10 (a validar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Seguimiento de un caso derivado a Servicio Técnico</t>
         </is>
       </c>
-      <c r="C13" s="19" t="inlineStr">
+      <c r="C14" s="19" t="inlineStr">
         <is>
           <t>Servicio Técnico</t>
         </is>
       </c>
-      <c r="D13" s="20" t="inlineStr">
+      <c r="D14" s="20" t="inlineStr">
         <is>
           <t>A DEFINIR</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Estado de la resolución y plazo estimado</t>
         </is>
       </c>
-      <c r="F13" s="28" t="inlineStr">
+      <c r="F14" s="28" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G13" s="17" t="inlineStr">
+      <c r="G14" s="17" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="H13" s="17" t="inlineStr">
+      <c r="H14" s="17" t="inlineStr">
         <is>
           <t>Cierra el reclamo con la conformidad del cliente. SLA a definir.</t>
         </is>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15" ht="30" customHeight="1" s="13">
-      <c r="A15" s="22" t="inlineStr">
+    <row r="15" ht="30" customHeight="1" s="13"/>
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>Estado de validación: Pendiente = relevamiento del hito aún no iniciado (responsable tomado del documento de relevamiento)   |   En proceso = relevamiento en curso: reuniones con las áreas y minutas   |   Validado = relevamiento realizado, reuniones con sus minutas y validación formal del sector</t>
         </is>
@@ -1692,7 +1740,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="39.6" customHeight="1" s="13">
+    <row r="15" ht="92" customHeight="1" s="13">
       <c r="A15" s="2" t="n">
         <v>11</v>
       </c>
@@ -1701,29 +1749,29 @@
           <t>Escalación de un pendiente del acta no resuelto en el plazo acordado</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>A DEFINIR</t>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="E15" s="29" t="inlineStr">
+        <is>
+          <t>Apoya</t>
+        </is>
+      </c>
+      <c r="F15" s="29" t="inlineStr">
+        <is>
+          <t>Apoya</t>
+        </is>
+      </c>
+      <c r="G15" s="24" t="inlineStr">
+        <is>
+          <t>Responsable</t>
         </is>
       </c>
       <c r="H15" s="28" t="inlineStr">
@@ -1733,12 +1781,12 @@
       </c>
       <c r="I15" s="17" t="inlineStr">
         <is>
-          <t>— (no relevado)</t>
+          <t>11 (excepción posterior a la 10)</t>
         </is>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>No surge del relevamiento; definir con Instalaciones, Servicio Técnico y Posventa.</t>
+          <t>Propuesta 07/10 (a validar). Se activa cuando un pendiente del acta (hito 7) vence sin resolverse. Posventa lo detecta y lo escala al jefe del área dueña del pendiente (Instalaciones o Servicio Técnico), que lo resuelve con un nuevo plazo; si vuelve a vencer, se escala a la Gerencia de Operaciones. Posventa informa al cliente el escalamiento y el nuevo plazo, y confirma el cierre. Equivale a un SLA con regla de escalamiento, como el hito 12. Reuniones: R1 (planteado).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Quitar hito cierre de instalacion
</commit_message>
<xml_diff>
--- a/assets/procesos/nuevos-clientes-instalacion/matrices-responsabilidades.xlsx
+++ b/assets/procesos/nuevos-clientes-instalacion/matrices-responsabilidades.xlsx
@@ -664,7 +664,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Proceso: "Nuevos clientes con instalación de alarmas y/o cámaras"</t>
+          <t>Proceso: "Nuevos clientes con alarmas y/o cámaras: del primer contacto a la posventa"</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
     </row>
     <row r="9" ht="39.6" customHeight="1" s="13">
       <c r="A9" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
@@ -920,7 +920,7 @@
     </row>
     <row r="10" ht="39.6" customHeight="1" s="13">
       <c r="A10" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
@@ -960,7 +960,7 @@
     </row>
     <row r="11" ht="58" customHeight="1" s="13">
       <c r="A11" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
     </row>
     <row r="12" ht="39.6" customHeight="1" s="13">
       <c r="A12" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="13" ht="40" customHeight="1" s="13">
       <c r="A13" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -1080,7 +1080,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
@@ -1119,7 +1119,7 @@
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" s="13"/>
-    <row r="16">
+    <row r="16" ht="30" customHeight="1" s="13">
       <c r="A16" s="22" t="inlineStr">
         <is>
           <t>Estado de validación: Pendiente = relevamiento del hito aún no iniciado (responsable tomado del documento de relevamiento)   |   En proceso = relevamiento en curso: reuniones con las áreas y minutas   |   Validado = relevamiento realizado, reuniones con sus minutas y validación formal del sector</t>
@@ -1128,10 +1128,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A15:H15"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F13">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
@@ -1160,7 +1160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" style="13" min="1" max="1"/>
@@ -1185,7 +1185,7 @@
     <row r="2" ht="16.05" customHeight="1" s="13">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Proceso: "Nuevos clientes con instalación de alarmas y/o cámaras"</t>
+          <t>Proceso: "Nuevos clientes con alarmas y/o cámaras: del primer contacto a la posventa"</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Ejecución de la instalación</t>
+          <t>Cierre de la instalación y firma del acta de conformidad</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -1500,30 +1500,30 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Cierre de la instalación y firma del acta de conformidad</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
+          <t>Registro de pendientes en el acta con responsable y plazo asignado</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="E10" s="24" t="inlineStr">
         <is>
           <t>Responsable</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="F10" s="25" t="inlineStr">
+        <is>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="inlineStr">
         <is>
           <t>No participa</t>
         </is>
@@ -1535,10 +1535,14 @@
       </c>
       <c r="I10" s="17" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="J10" s="17" t="n"/>
+          <t>10 (inferido)</t>
+        </is>
+      </c>
+      <c r="J10" s="17" t="inlineStr">
+        <is>
+          <t>Hoy el acta no asigna responsable ni plazo. Instalaciones cierra el acta; la asignación de responsable/plazo no está relevada.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="39.6" customHeight="1" s="13">
       <c r="A11" s="2" t="n">
@@ -1546,7 +1550,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Registro de pendientes en el acta con responsable y plazo asignado</t>
+          <t>Comunicación de finalización / activación del sistema al cliente</t>
         </is>
       </c>
       <c r="C11" s="23" t="inlineStr">
@@ -1564,16 +1568,16 @@
           <t>Responsable</t>
         </is>
       </c>
-      <c r="F11" s="25" t="inlineStr">
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="G11" s="25" t="inlineStr">
         <is>
           <t>Informado</t>
         </is>
       </c>
-      <c r="G11" s="23" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
       <c r="H11" s="28" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -1581,49 +1585,49 @@
       </c>
       <c r="I11" s="17" t="inlineStr">
         <is>
-          <t>10 (inferido)</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J11" s="17" t="inlineStr">
         <is>
-          <t>Hoy el acta no asigna responsable ni plazo. Instalaciones cierra el acta; la asignación de responsable/plazo no está relevada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="39.6" customHeight="1" s="13">
+          <t>Instalaciones da de alta el sistema en la central y capacita al cliente; Posventa valida luego el funcionamiento. Reuniones: R1 (tratado, sin cierre).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1" s="13">
       <c r="A12" s="2" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Comunicación de finalización / activación del sistema al cliente</t>
-        </is>
-      </c>
-      <c r="C12" s="23" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="D12" s="23" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="E12" s="24" t="inlineStr">
+          <t>Control de calidad y encuesta de satisfacción</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>Responsable</t>
         </is>
       </c>
-      <c r="F12" s="23" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="G12" s="25" t="inlineStr">
-        <is>
-          <t>Informado</t>
-        </is>
-      </c>
       <c r="H12" s="28" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -1631,45 +1635,45 @@
       </c>
       <c r="I12" s="17" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J12" s="17" t="inlineStr">
         <is>
-          <t>Instalaciones da de alta el sistema en la central y capacita al cliente; Posventa valida luego el funcionamiento. Reuniones: R1 (tratado, sin cierre).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="58" customHeight="1" s="13">
+          <t>La bienvenida es la etapa 8, a cargo de Atención al Cliente (antes de la instalación). Este hito corresponde a la etapa 11, control de calidad posterior a la instalación (Posventa).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="39.6" customHeight="1" s="13">
       <c r="A13" s="2" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Control de calidad y encuesta de satisfacción</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
+          <t>Clasificación y canalización de reclamos según tipo (comercial / técnico / servicio)</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="D13" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="E13" s="23" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="F13" s="25" t="inlineStr">
+        <is>
+          <t>Informado</t>
+        </is>
+      </c>
+      <c r="G13" s="24" t="inlineStr">
         <is>
           <t>Responsable</t>
         </is>
@@ -1681,22 +1685,22 @@
       </c>
       <c r="I13" s="17" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>11 / 13</t>
         </is>
       </c>
       <c r="J13" s="17" t="inlineStr">
         <is>
-          <t>La bienvenida es la etapa 8, a cargo de Atención al Cliente (antes de la instalación). Este hito corresponde a la etapa 11, control de calidad posterior a la instalación (Posventa).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="39.6" customHeight="1" s="13">
+          <t>Posventa canaliza a Servicio Técnico las fallas del período inicial. El relevamiento no define reclamos comerciales ni de servicio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="92" customHeight="1" s="13">
       <c r="A14" s="2" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Clasificación y canalización de reclamos según tipo (comercial / técnico / servicio)</t>
+          <t>Escalación de un pendiente del acta no resuelto en el plazo acordado</t>
         </is>
       </c>
       <c r="C14" s="23" t="inlineStr">
@@ -1709,14 +1713,14 @@
           <t>No participa</t>
         </is>
       </c>
-      <c r="E14" s="23" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="F14" s="25" t="inlineStr">
-        <is>
-          <t>Informado</t>
+      <c r="E14" s="29" t="inlineStr">
+        <is>
+          <t>Apoya</t>
+        </is>
+      </c>
+      <c r="F14" s="29" t="inlineStr">
+        <is>
+          <t>Apoya</t>
         </is>
       </c>
       <c r="G14" s="24" t="inlineStr">
@@ -1731,49 +1735,49 @@
       </c>
       <c r="I14" s="17" t="inlineStr">
         <is>
-          <t>11 / 13</t>
+          <t>11 (excepción posterior a la 10)</t>
         </is>
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>Posventa canaliza a Servicio Técnico las fallas del período inicial. El relevamiento no define reclamos comerciales ni de servicio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="92" customHeight="1" s="13">
+          <t>Propuesta 07/10 (a validar). Se activa cuando un pendiente del acta (hito 6) vence sin resolverse. Posventa lo detecta y lo escala al jefe del área dueña del pendiente (Instalaciones o Servicio Técnico), que lo resuelve con un nuevo plazo; si vuelve a vencer, se escala a la Gerencia de Operaciones. Posventa informa al cliente el escalamiento y el nuevo plazo, y confirma el cierre. Equivale a un SLA con regla de escalamiento, como el hito 11. Reuniones: R1 (planteado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="39.6" customHeight="1" s="13">
       <c r="A15" s="2" t="n">
         <v>11</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Escalación de un pendiente del acta no resuelto en el plazo acordado</t>
-        </is>
-      </c>
-      <c r="C15" s="23" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="D15" s="23" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="E15" s="29" t="inlineStr">
+          <t>Resolución de un caso técnico derivado por Posventa (dentro de un SLA)</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>No participa</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
         <is>
           <t>Apoya</t>
         </is>
       </c>
-      <c r="F15" s="29" t="inlineStr">
-        <is>
-          <t>Apoya</t>
-        </is>
-      </c>
-      <c r="G15" s="24" t="inlineStr">
-        <is>
-          <t>Responsable</t>
-        </is>
-      </c>
       <c r="H15" s="28" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -1781,12 +1785,12 @@
       </c>
       <c r="I15" s="17" t="inlineStr">
         <is>
-          <t>11 (excepción posterior a la 10)</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>Propuesta 07/10 (a validar). Se activa cuando un pendiente del acta (hito 7) vence sin resolverse. Posventa lo detecta y lo escala al jefe del área dueña del pendiente (Instalaciones o Servicio Técnico), que lo resuelve con un nuevo plazo; si vuelve a vencer, se escala a la Gerencia de Operaciones. Posventa informa al cliente el escalamiento y el nuevo plazo, y confirma el cierre. Equivale a un SLA con regla de escalamiento, como el hito 12. Reuniones: R1 (planteado).</t>
+          <t>Responsables definidos; falta definir el SLA.</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1800,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Resolución de un caso técnico derivado por Posventa (dentro de un SLA)</t>
+          <t>Resolución de una situación administrativa derivada por Posventa (ej. saldo de deuda)</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -1804,9 +1808,9 @@
           <t>No participa</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Responsable</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -1814,9 +1818,9 @@
           <t>No participa</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>Responsable</t>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>No participa</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
@@ -1831,77 +1835,28 @@
       </c>
       <c r="I16" s="17" t="inlineStr">
         <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="J16" s="17" t="inlineStr">
-        <is>
-          <t>Responsables definidos; falta definir el SLA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="39.6" customHeight="1" s="13">
-      <c r="A17" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Resolución de una situación administrativa derivada por Posventa (ej. saldo de deuda)</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>Responsable</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>No participa</t>
-        </is>
-      </c>
-      <c r="G17" s="11" t="inlineStr">
-        <is>
-          <t>Apoya</t>
-        </is>
-      </c>
-      <c r="H17" s="28" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I17" s="17" t="inlineStr">
-        <is>
           <t>15</t>
         </is>
       </c>
-      <c r="J17" s="17" t="n"/>
-    </row>
-    <row r="18"/>
-    <row r="19" ht="30" customHeight="1" s="13">
-      <c r="A19" s="22" t="inlineStr">
+      <c r="J16" s="17" t="n"/>
+    </row>
+    <row r="17" s="13"/>
+    <row r="18" ht="30" customHeight="1" s="13">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>Estado de validación: Pendiente = relevamiento del hito aún no iniciado (responsable tomado del documento de relevamiento)   |   En proceso = relevamiento en curso: reuniones con las áreas y minutas   |   Validado = relevamiento realizado, reuniones con sus minutas y validación formal del sector</t>
         </is>
       </c>
     </row>
+    <row r="19" s="13"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A19:J19"/>
+    <mergeCell ref="A18:J18"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H17">
+  <conditionalFormatting sqref="H5:H16">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pendiente"</formula>
     </cfRule>
@@ -1913,7 +1868,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendiente,En proceso,Validado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>